<commit_message>
add modulo 2- word search
</commit_message>
<xml_diff>
--- a/01-essentials/material_curso/modulo-02/W02_Word-Search.xlsx
+++ b/01-essentials/material_curso/modulo-02/W02_Word-Search.xlsx
@@ -1,20 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18201"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC95A56E-53D6-4A95-9D22-7FB329F35BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Word search" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="57">
   <si>
     <t>Q</t>
   </si>
@@ -225,11 +240,14 @@
   <si>
     <t>J1:J9</t>
   </si>
+  <si>
+    <t>H13:N13</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -298,182 +316,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="50">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="25">
     <dxf>
       <fill>
         <patternFill>
@@ -958,24 +801,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V26"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="2.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="2.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="2.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="2.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="2.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="2.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="2.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1035,7 +875,7 @@
       </c>
       <c r="V1" s="4"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1088,7 +928,7 @@
       <c r="U2" s="4"/>
       <c r="V2" s="4"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -1143,7 +983,7 @@
       <c r="U3" s="4"/>
       <c r="V3" s="4"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -1192,11 +1032,13 @@
       <c r="Q4" t="s">
         <v>28</v>
       </c>
-      <c r="R4" s="1"/>
+      <c r="R4" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="U4" s="4"/>
       <c r="V4" s="4"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -1249,7 +1091,7 @@
       <c r="U5" s="4"/>
       <c r="V5" s="4"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -1302,7 +1144,7 @@
       <c r="U6" s="4"/>
       <c r="V6" s="4"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -1355,7 +1197,7 @@
       <c r="U7" s="4"/>
       <c r="V7" s="4"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
@@ -1408,7 +1250,7 @@
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1461,7 +1303,7 @@
       <c r="U9" s="4"/>
       <c r="V9" s="4"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
@@ -1514,7 +1356,7 @@
       <c r="U10" s="4"/>
       <c r="V10" s="4"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>0</v>
       </c>
@@ -1567,7 +1409,7 @@
       <c r="U11" s="4"/>
       <c r="V11" s="4"/>
     </row>
-    <row r="12" spans="1:22" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>25</v>
       </c>
@@ -1620,7 +1462,7 @@
       <c r="U12" s="4"/>
       <c r="V12" s="4"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -1673,7 +1515,7 @@
       <c r="U13" s="4"/>
       <c r="V13" s="4"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
@@ -1726,7 +1568,7 @@
       <c r="U14" s="4"/>
       <c r="V14" s="4"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>4</v>
       </c>
@@ -1779,67 +1621,67 @@
       <c r="U15" s="4"/>
       <c r="V15" s="4"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="Q16" t="s">
         <v>40</v>
       </c>
       <c r="R16" s="1"/>
     </row>
-    <row r="17" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q17" t="s">
         <v>41</v>
       </c>
       <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q18" t="s">
         <v>42</v>
       </c>
       <c r="R18" s="1"/>
     </row>
-    <row r="19" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q19" t="s">
         <v>43</v>
       </c>
       <c r="R19" s="1"/>
     </row>
-    <row r="20" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q20" t="s">
         <v>44</v>
       </c>
       <c r="R20" s="1"/>
     </row>
-    <row r="21" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q21" t="s">
         <v>45</v>
       </c>
       <c r="R21" s="1"/>
     </row>
-    <row r="22" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q22" t="s">
         <v>46</v>
       </c>
       <c r="R22" s="1"/>
     </row>
-    <row r="23" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q23" t="s">
         <v>47</v>
       </c>
       <c r="R23" s="1"/>
     </row>
-    <row r="24" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q24" t="s">
         <v>48</v>
       </c>
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q25" t="s">
         <v>49</v>
       </c>
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="17:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q26" t="s">
         <v>50</v>
       </c>
@@ -1850,127 +1692,127 @@
     <mergeCell ref="U1:V15"/>
   </mergeCells>
   <conditionalFormatting sqref="S3">
-    <cfRule type="expression" dxfId="0" priority="60" stopIfTrue="1">
+    <cfRule type="expression" dxfId="24" priority="60" stopIfTrue="1">
       <formula>UPPER(R3)="J1:J9"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S4">
-    <cfRule type="expression" dxfId="24" priority="61" stopIfTrue="1">
+    <cfRule type="expression" dxfId="23" priority="61" stopIfTrue="1">
       <formula>UPPER(R4)="H13:N13"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S5">
-    <cfRule type="expression" dxfId="23" priority="62" stopIfTrue="1">
+    <cfRule type="expression" dxfId="22" priority="62" stopIfTrue="1">
       <formula>UPPER(R5)="D2:D4"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S6">
-    <cfRule type="expression" dxfId="22" priority="63" stopIfTrue="1">
+    <cfRule type="expression" dxfId="21" priority="63" stopIfTrue="1">
       <formula>UPPER(R6)="C8:H8"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S7">
-    <cfRule type="expression" dxfId="21" priority="64" stopIfTrue="1">
+    <cfRule type="expression" dxfId="20" priority="64" stopIfTrue="1">
       <formula>UPPER(R7)="B6:B9"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S8">
-    <cfRule type="expression" dxfId="20" priority="65" stopIfTrue="1">
+    <cfRule type="expression" dxfId="19" priority="65" stopIfTrue="1">
       <formula>UPPER(R8)="I12:M12"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S9">
-    <cfRule type="expression" dxfId="19" priority="66" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="66" stopIfTrue="1">
       <formula>UPPER(R9)="N3:N8"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S11">
-    <cfRule type="expression" dxfId="18" priority="67" stopIfTrue="1">
+    <cfRule type="expression" dxfId="17" priority="67" stopIfTrue="1">
       <formula>UPPER(R11)="K11:O11"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S10">
-    <cfRule type="expression" dxfId="17" priority="68" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="68" stopIfTrue="1">
       <formula>UPPER(R10)="M3:M6"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S12">
-    <cfRule type="expression" dxfId="16" priority="69" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="69" stopIfTrue="1">
       <formula>UPPER(R12)="A12:A15"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S13">
-    <cfRule type="expression" dxfId="15" priority="70" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="70" stopIfTrue="1">
       <formula>UPPER(R13)="F7:K7"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S14">
-    <cfRule type="expression" dxfId="14" priority="71" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="71" stopIfTrue="1">
       <formula>UPPER(R14)="G6:M6"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S15">
-    <cfRule type="expression" dxfId="13" priority="72" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="72" stopIfTrue="1">
       <formula>UPPER(R15)="L1:L5"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S16">
-    <cfRule type="expression" dxfId="12" priority="73" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="73" stopIfTrue="1">
       <formula>UPPER(R16)="D10:G10"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S17">
-    <cfRule type="expression" dxfId="11" priority="74" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="74" stopIfTrue="1">
       <formula>UPPER(R17)="I1:N1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S18">
-    <cfRule type="expression" dxfId="10" priority="75" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="75" stopIfTrue="1">
       <formula>UPPER(R18)="F15:H15"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S19">
-    <cfRule type="expression" dxfId="9" priority="76" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="76" stopIfTrue="1">
       <formula>UPPER(R19)="I3:K3"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S20">
-    <cfRule type="expression" dxfId="8" priority="77" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="77" stopIfTrue="1">
       <formula>UPPER(R20)="K9:M9"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S21">
-    <cfRule type="expression" dxfId="7" priority="78" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="78" stopIfTrue="1">
       <formula>UPPER(R21)="F9:J9"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S22">
-    <cfRule type="expression" dxfId="6" priority="79" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="79" stopIfTrue="1">
       <formula>UPPER(R22)="H14:O14"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S23">
-    <cfRule type="expression" dxfId="5" priority="80" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="80" stopIfTrue="1">
       <formula>UPPER(R23)="K10:M10"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S24">
-    <cfRule type="expression" dxfId="4" priority="81" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="81" stopIfTrue="1">
       <formula>UPPER(R24)="E2:I2"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S25">
-    <cfRule type="expression" dxfId="3" priority="82" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="82" stopIfTrue="1">
       <formula>UPPER(R25)="B11:E11"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S26">
-    <cfRule type="expression" dxfId="2" priority="83" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="83" stopIfTrue="1">
       <formula>UPPER(R26)="A3:A5"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2">
-    <cfRule type="expression" dxfId="1" priority="59" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="59" stopIfTrue="1">
       <formula>UPPER(R2)="O7:O14"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>